<commit_message>
daily market data update and gold signal check
</commit_message>
<xml_diff>
--- a/gold_beneficiaries_year_by_year.xlsx
+++ b/gold_beneficiaries_year_by_year.xlsx
@@ -875,37 +875,37 @@
         <v>21</v>
       </c>
       <c r="J6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="K6" t="n">
         <v>52.5</v>
       </c>
       <c r="L6" t="n">
-        <v>3.47</v>
+        <v>2.26</v>
       </c>
       <c r="M6" t="n">
-        <v>2.07</v>
+        <v>2.34</v>
       </c>
       <c r="N6" t="n">
         <v>44.99</v>
       </c>
       <c r="O6" t="n">
-        <v>-12.86</v>
+        <v>-57.48</v>
       </c>
       <c r="P6" t="n">
         <v>40000000</v>
       </c>
       <c r="Q6" t="n">
-        <v>1389650</v>
+        <v>905789</v>
       </c>
       <c r="R6" t="n">
-        <v>3106391</v>
+        <v>1438401</v>
       </c>
       <c r="S6" t="n">
-        <v>210.64</v>
+        <v>43.84</v>
       </c>
       <c r="T6" t="n">
-        <v>2.27</v>
+        <v>1.54</v>
       </c>
       <c r="U6" s="1" t="n">
         <v>41165</v>
@@ -1008,10 +1008,10 @@
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>-57.48</v>
       </c>
       <c r="F2" t="n">
-        <v>1000000</v>
+        <v>425200</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -1023,13 +1023,13 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>-57.48</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>-57.48</v>
       </c>
       <c r="L2" t="n">
-        <v>0</v>
+        <v>-57.48</v>
       </c>
     </row>
     <row r="3">
@@ -1050,10 +1050,10 @@
         <v>4</v>
       </c>
       <c r="E3" t="n">
-        <v>6.6</v>
+        <v>6.59</v>
       </c>
       <c r="F3" t="n">
-        <v>1065992</v>
+        <v>453209</v>
       </c>
       <c r="G3" t="n">
         <v>2</v>
@@ -1071,7 +1071,7 @@
         <v>13.22</v>
       </c>
       <c r="L3" t="n">
-        <v>-10.62</v>
+        <v>-10.63</v>
       </c>
     </row>
     <row r="4">
@@ -1095,7 +1095,7 @@
         <v>4.73</v>
       </c>
       <c r="F4" t="n">
-        <v>1116462</v>
+        <v>474667</v>
       </c>
       <c r="G4" t="n">
         <v>2</v>
@@ -1134,10 +1134,10 @@
         <v>3</v>
       </c>
       <c r="E5" t="n">
-        <v>-17.47</v>
+        <v>-17.49</v>
       </c>
       <c r="F5" t="n">
-        <v>921379</v>
+        <v>391635</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -1149,13 +1149,13 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>-6.09</v>
+        <v>-6.1</v>
       </c>
       <c r="K5" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>-11.08</v>
+        <v>-11.12</v>
       </c>
     </row>
     <row r="6">
@@ -1179,7 +1179,7 @@
         <v>-3.17</v>
       </c>
       <c r="F6" t="n">
-        <v>892168</v>
+        <v>379218</v>
       </c>
       <c r="G6" t="n">
         <v>2</v>
@@ -1221,7 +1221,7 @@
         <v>-8</v>
       </c>
       <c r="F7" t="n">
-        <v>820794</v>
+        <v>348881</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -1260,10 +1260,10 @@
         <v>2</v>
       </c>
       <c r="E8" t="n">
-        <v>8.51</v>
+        <v>18.21</v>
       </c>
       <c r="F8" t="n">
-        <v>890679</v>
+        <v>412425</v>
       </c>
       <c r="G8" t="n">
         <v>2</v>
@@ -1275,13 +1275,13 @@
         <v>100</v>
       </c>
       <c r="J8" t="n">
-        <v>4.2</v>
+        <v>8.75</v>
       </c>
       <c r="K8" t="n">
+        <v>11.03</v>
+      </c>
+      <c r="L8" t="n">
         <v>6.47</v>
-      </c>
-      <c r="L8" t="n">
-        <v>1.92</v>
       </c>
     </row>
     <row r="9">
@@ -1305,7 +1305,7 @@
         <v>20.62</v>
       </c>
       <c r="F9" t="n">
-        <v>1074320</v>
+        <v>497459</v>
       </c>
       <c r="G9" t="n">
         <v>2</v>
@@ -1347,7 +1347,7 @@
         <v>-6.38</v>
       </c>
       <c r="F10" t="n">
-        <v>1005830</v>
+        <v>465745</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
@@ -1389,7 +1389,7 @@
         <v>42.82</v>
       </c>
       <c r="F11" t="n">
-        <v>1436477</v>
+        <v>665154</v>
       </c>
       <c r="G11" t="n">
         <v>1</v>
@@ -1431,7 +1431,7 @@
         <v>6.31</v>
       </c>
       <c r="F12" t="n">
-        <v>1527065</v>
+        <v>707101</v>
       </c>
       <c r="G12" t="n">
         <v>2</v>
@@ -1473,7 +1473,7 @@
         <v>10.64</v>
       </c>
       <c r="F13" t="n">
-        <v>1689492</v>
+        <v>782312</v>
       </c>
       <c r="G13" t="n">
         <v>2</v>
@@ -1515,7 +1515,7 @@
         <v>58.31</v>
       </c>
       <c r="F14" t="n">
-        <v>2674695</v>
+        <v>1238506</v>
       </c>
       <c r="G14" t="n">
         <v>5</v>
@@ -1557,7 +1557,7 @@
         <v>16.14</v>
       </c>
       <c r="F15" t="n">
-        <v>3106391</v>
+        <v>1438401</v>
       </c>
       <c r="G15" t="n">
         <v>1</v>
@@ -4077,25 +4077,25 @@
         <v>41179</v>
       </c>
       <c r="G2" t="n">
-        <v>1350</v>
+        <v>2666.926513671875</v>
       </c>
       <c r="H2" t="n">
-        <v>1350</v>
+        <v>1133.96875</v>
       </c>
       <c r="I2" t="n">
         <v>1000000</v>
       </c>
       <c r="J2" t="n">
-        <v>740.74</v>
+        <v>374.96</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>-57.48</v>
       </c>
       <c r="L2" t="n">
-        <v>0</v>
+        <v>-574803</v>
       </c>
       <c r="M2" t="n">
-        <v>1000000</v>
+        <v>425197</v>
       </c>
     </row>
     <row r="3">
@@ -4122,16 +4122,16 @@
         <v>41408</v>
       </c>
       <c r="G3" t="n">
-        <v>1370</v>
+        <v>1150.768310546875</v>
       </c>
       <c r="H3" t="n">
-        <v>1350</v>
+        <v>1133.96875</v>
       </c>
       <c r="I3" t="n">
         <v>1000000</v>
       </c>
       <c r="J3" t="n">
-        <v>729.9299999999999</v>
+        <v>868.98</v>
       </c>
       <c r="K3" t="n">
         <v>-1.46</v>
@@ -4167,25 +4167,25 @@
         <v>41481</v>
       </c>
       <c r="G4" t="n">
-        <v>1160</v>
+        <v>974.3731689453125</v>
       </c>
       <c r="H4" t="n">
-        <v>1240</v>
+        <v>1041.5712890625</v>
       </c>
       <c r="I4" t="n">
         <v>1000000</v>
       </c>
       <c r="J4" t="n">
-        <v>862.0700000000001</v>
+        <v>1026.3</v>
       </c>
       <c r="K4" t="n">
         <v>6.9</v>
       </c>
       <c r="L4" t="n">
-        <v>68966</v>
+        <v>68965</v>
       </c>
       <c r="M4" t="n">
-        <v>1068966</v>
+        <v>1068965</v>
       </c>
     </row>
     <row r="5">
@@ -4212,16 +4212,16 @@
         <v>41520</v>
       </c>
       <c r="G5" t="n">
-        <v>1210</v>
+        <v>1016.372009277344</v>
       </c>
       <c r="H5" t="n">
-        <v>1370</v>
+        <v>1150.768310546875</v>
       </c>
       <c r="I5" t="n">
         <v>1000000</v>
       </c>
       <c r="J5" t="n">
-        <v>826.45</v>
+        <v>983.89</v>
       </c>
       <c r="K5" t="n">
         <v>13.22</v>
@@ -4257,19 +4257,19 @@
         <v>41589</v>
       </c>
       <c r="G6" t="n">
-        <v>1600</v>
+        <v>1343.963012695312</v>
       </c>
       <c r="H6" t="n">
-        <v>1430</v>
+        <v>1201.166870117188</v>
       </c>
       <c r="I6" t="n">
         <v>1000000</v>
       </c>
       <c r="J6" t="n">
-        <v>625</v>
+        <v>744.0700000000001</v>
       </c>
       <c r="K6" t="n">
-        <v>-10.62</v>
+        <v>-10.63</v>
       </c>
       <c r="L6" t="n">
         <v>-106250</v>
@@ -4302,25 +4302,25 @@
         <v>41698</v>
       </c>
       <c r="G7" t="n">
-        <v>853</v>
+        <v>852.5764770507812</v>
       </c>
       <c r="H7" t="n">
-        <v>874</v>
+        <v>873.575927734375</v>
       </c>
       <c r="I7" t="n">
         <v>1000000</v>
       </c>
       <c r="J7" t="n">
-        <v>1172.33</v>
+        <v>1172.92</v>
       </c>
       <c r="K7" t="n">
         <v>2.46</v>
       </c>
       <c r="L7" t="n">
-        <v>24619</v>
+        <v>24631</v>
       </c>
       <c r="M7" t="n">
-        <v>1024619</v>
+        <v>1024631</v>
       </c>
     </row>
     <row r="8">
@@ -4347,16 +4347,16 @@
         <v>41824</v>
       </c>
       <c r="G8" t="n">
-        <v>945</v>
+        <v>944.9739379882812</v>
       </c>
       <c r="H8" t="n">
-        <v>966</v>
+        <v>965.973388671875</v>
       </c>
       <c r="I8" t="n">
         <v>1000000</v>
       </c>
       <c r="J8" t="n">
-        <v>1058.2</v>
+        <v>1058.23</v>
       </c>
       <c r="K8" t="n">
         <v>2.22</v>
@@ -4392,22 +4392,22 @@
         <v>42033</v>
       </c>
       <c r="G9" t="n">
-        <v>899</v>
+        <v>898.7752075195312</v>
       </c>
       <c r="H9" t="n">
-        <v>899</v>
+        <v>898.7752075195312</v>
       </c>
       <c r="I9" t="n">
         <v>1000000</v>
       </c>
       <c r="J9" t="n">
-        <v>1112.35</v>
+        <v>1112.63</v>
       </c>
       <c r="K9" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="M9" t="n">
         <v>1000000</v>
@@ -4437,25 +4437,25 @@
         <v>42250</v>
       </c>
       <c r="G10" t="n">
-        <v>445</v>
+        <v>445.187744140625</v>
       </c>
       <c r="H10" t="n">
-        <v>413</v>
+        <v>413.2686157226562</v>
       </c>
       <c r="I10" t="n">
         <v>1000000</v>
       </c>
       <c r="J10" t="n">
-        <v>2247.19</v>
+        <v>2246.24</v>
       </c>
       <c r="K10" t="n">
-        <v>-7.19</v>
+        <v>-7.17</v>
       </c>
       <c r="L10" t="n">
-        <v>-71910</v>
+        <v>-71698</v>
       </c>
       <c r="M10" t="n">
-        <v>928090</v>
+        <v>928302</v>
       </c>
     </row>
     <row r="11">
@@ -4482,7 +4482,7 @@
         <v>42306</v>
       </c>
       <c r="G11" t="n">
-        <v>424</v>
+        <v>424.1883239746094</v>
       </c>
       <c r="H11" t="n">
         <v>377</v>
@@ -4491,16 +4491,16 @@
         <v>1000000</v>
       </c>
       <c r="J11" t="n">
-        <v>2358.49</v>
+        <v>2357.44</v>
       </c>
       <c r="K11" t="n">
-        <v>-11.08</v>
+        <v>-11.12</v>
       </c>
       <c r="L11" t="n">
-        <v>-110849</v>
+        <v>-111244</v>
       </c>
       <c r="M11" t="n">
-        <v>889151</v>
+        <v>888756</v>
       </c>
     </row>
     <row r="12">
@@ -4701,31 +4701,31 @@
         <v>5.03</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>43626</v>
+        <v>43622</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>43640</v>
+        <v>43636</v>
       </c>
       <c r="G16" t="n">
-        <v>780</v>
+        <v>725</v>
       </c>
       <c r="H16" t="n">
-        <v>795</v>
+        <v>805</v>
       </c>
       <c r="I16" t="n">
         <v>1000000</v>
       </c>
       <c r="J16" t="n">
-        <v>1282.05</v>
+        <v>1379.31</v>
       </c>
       <c r="K16" t="n">
-        <v>1.92</v>
+        <v>11.03</v>
       </c>
       <c r="L16" t="n">
-        <v>19231</v>
+        <v>110345</v>
       </c>
       <c r="M16" t="n">
-        <v>1019231</v>
+        <v>1110345</v>
       </c>
     </row>
     <row r="17">

</xml_diff>